<commit_message>
update pr template f7defe4831d2704cbc89ab312f42237fe7facb4d
</commit_message>
<xml_diff>
--- a/main/ig/StructureDefinition-fr-core-observation-bmi.xlsx
+++ b/main/ig/StructureDefinition-fr-core-observation-bmi.xlsx
@@ -60,7 +60,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2024-05-23T14:35:00+00:00</t>
+    <t>2024-06-11T15:33:12+00:00</t>
   </si>
   <si>
     <t>Publisher</t>
@@ -13303,7 +13303,7 @@
         <v>83</v>
       </c>
       <c r="X90" t="s" s="2">
-        <v>248</v>
+        <v>158</v>
       </c>
       <c r="Y90" t="s" s="2">
         <v>658</v>

</xml_diff>